<commit_message>
Daily recap, matchup updates, learning and research 2026-08-24
</commit_message>
<xml_diff>
--- a/data/k-props/2026-08-24.xlsx
+++ b/data/k-props/2026-08-24.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="84">
   <si>
     <t>date</t>
   </si>
@@ -145,15 +145,21 @@
     <t>lineup_unweighted_30d_posted</t>
   </si>
   <si>
+    <t>U</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>&lt;6</t>
+  </si>
+  <si>
+    <t>Framber Valdez</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>&lt;6</t>
-  </si>
-  <si>
-    <t>Framber Valdez</t>
-  </si>
-  <si>
     <t>Ranger Suarez</t>
   </si>
   <si>
@@ -163,6 +169,9 @@
     <t>Sandy Alcantara</t>
   </si>
   <si>
+    <t>O</t>
+  </si>
+  <si>
     <t>Ryan Feltner</t>
   </si>
   <si>
@@ -185,6 +194,9 @@
   </si>
   <si>
     <t>Opener / bullpen game</t>
+  </si>
+  <si>
+    <t>L</t>
   </si>
   <si>
     <t>Parker Messick</t>
@@ -832,17 +844,23 @@
       <c r="Y2">
         <v>0.8829</v>
       </c>
+      <c r="Z2">
+        <v>5</v>
+      </c>
       <c r="AA2" t="s">
         <v>44</v>
       </c>
+      <c r="AB2">
+        <v>-0.99</v>
+      </c>
       <c r="AC2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD2">
         <v>4.51</v>
       </c>
       <c r="AE2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF2">
         <v>0.2669</v>
@@ -852,6 +870,18 @@
       </c>
       <c r="AH2">
         <v>0</v>
+      </c>
+      <c r="AI2">
+        <v>0.49</v>
+      </c>
+      <c r="AJ2">
+        <v>0.49</v>
+      </c>
+      <c r="AK2">
+        <v>0.49</v>
+      </c>
+      <c r="AL2">
+        <v>0.49</v>
       </c>
       <c r="AM2">
         <v>4.51</v>
@@ -862,7 +892,7 @@
         <v>39</v>
       </c>
       <c r="B3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C3">
         <v>3.5</v>
@@ -933,17 +963,23 @@
       <c r="Y3">
         <v>0.88</v>
       </c>
+      <c r="Z3">
+        <v>0</v>
+      </c>
       <c r="AA3" t="s">
         <v>44</v>
       </c>
+      <c r="AB3">
+        <v>-0.53</v>
+      </c>
       <c r="AC3" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD3">
         <v>2.97</v>
       </c>
       <c r="AE3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF3">
         <v>0.1599</v>
@@ -953,6 +989,18 @@
       </c>
       <c r="AH3">
         <v>0</v>
+      </c>
+      <c r="AI3">
+        <v>-2.97</v>
+      </c>
+      <c r="AJ3">
+        <v>2.97</v>
+      </c>
+      <c r="AK3">
+        <v>-2.97</v>
+      </c>
+      <c r="AL3">
+        <v>2.97</v>
       </c>
       <c r="AM3">
         <v>2.97</v>
@@ -963,7 +1011,7 @@
         <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C4">
         <v>4.5</v>
@@ -975,7 +1023,7 @@
         <v>110</v>
       </c>
       <c r="F4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G4">
         <v>823828</v>
@@ -1034,17 +1082,23 @@
       <c r="Y4">
         <v>0.916</v>
       </c>
+      <c r="Z4">
+        <v>4</v>
+      </c>
       <c r="AA4" t="s">
         <v>44</v>
       </c>
+      <c r="AB4">
+        <v>-0.53</v>
+      </c>
       <c r="AC4" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD4">
         <v>3.97</v>
       </c>
       <c r="AE4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF4">
         <v>0.2055</v>
@@ -1054,6 +1108,18 @@
       </c>
       <c r="AH4">
         <v>0</v>
+      </c>
+      <c r="AI4">
+        <v>0.03</v>
+      </c>
+      <c r="AJ4">
+        <v>0.03</v>
+      </c>
+      <c r="AK4">
+        <v>0.03</v>
+      </c>
+      <c r="AL4">
+        <v>0.03</v>
       </c>
       <c r="AM4">
         <v>3.97</v>
@@ -1064,7 +1130,7 @@
         <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C5">
         <v>4.5</v>
@@ -1076,7 +1142,7 @@
         <v>-125</v>
       </c>
       <c r="F5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G5">
         <v>823828</v>
@@ -1135,17 +1201,23 @@
       <c r="Y5">
         <v>0.9965</v>
       </c>
+      <c r="Z5">
+        <v>6</v>
+      </c>
       <c r="AA5" t="s">
-        <v>44</v>
+        <v>52</v>
+      </c>
+      <c r="AB5">
+        <v>-0.45</v>
       </c>
       <c r="AC5" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD5">
         <v>4.05</v>
       </c>
       <c r="AE5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF5">
         <v>0.1753</v>
@@ -1155,6 +1227,18 @@
       </c>
       <c r="AH5">
         <v>0</v>
+      </c>
+      <c r="AI5">
+        <v>1.95</v>
+      </c>
+      <c r="AJ5">
+        <v>1.95</v>
+      </c>
+      <c r="AK5">
+        <v>1.95</v>
+      </c>
+      <c r="AL5">
+        <v>1.95</v>
       </c>
       <c r="AM5">
         <v>4.05</v>
@@ -1165,7 +1249,7 @@
         <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C6">
         <v>3.5</v>
@@ -1177,7 +1261,7 @@
         <v>-101</v>
       </c>
       <c r="F6" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="G6">
         <v>822695</v>
@@ -1236,17 +1320,23 @@
       <c r="Y6">
         <v>0.9728</v>
       </c>
+      <c r="Z6">
+        <v>6</v>
+      </c>
       <c r="AA6" t="s">
-        <v>44</v>
+        <v>52</v>
+      </c>
+      <c r="AB6">
+        <v>-0.54</v>
       </c>
       <c r="AC6" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD6">
         <v>2.96</v>
       </c>
       <c r="AE6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF6">
         <v>0.1467</v>
@@ -1256,6 +1346,18 @@
       </c>
       <c r="AH6">
         <v>0</v>
+      </c>
+      <c r="AI6">
+        <v>3.04</v>
+      </c>
+      <c r="AJ6">
+        <v>3.04</v>
+      </c>
+      <c r="AK6">
+        <v>3.04</v>
+      </c>
+      <c r="AL6">
+        <v>3.04</v>
       </c>
       <c r="AM6">
         <v>2.96</v>
@@ -1266,7 +1368,7 @@
         <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C7">
         <v>6.5</v>
@@ -1278,7 +1380,7 @@
         <v>-119</v>
       </c>
       <c r="F7" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="G7">
         <v>822695</v>
@@ -1337,17 +1439,23 @@
       <c r="Y7">
         <v>1.0261</v>
       </c>
+      <c r="Z7">
+        <v>7</v>
+      </c>
       <c r="AA7" t="s">
-        <v>44</v>
+        <v>52</v>
+      </c>
+      <c r="AB7">
+        <v>0.86</v>
       </c>
       <c r="AC7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD7">
         <v>7.36</v>
       </c>
       <c r="AE7" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="AF7">
         <v>0.2902</v>
@@ -1357,6 +1465,18 @@
       </c>
       <c r="AH7">
         <v>0</v>
+      </c>
+      <c r="AI7">
+        <v>-0.36</v>
+      </c>
+      <c r="AJ7">
+        <v>0.36</v>
+      </c>
+      <c r="AK7">
+        <v>-0.36</v>
+      </c>
+      <c r="AL7">
+        <v>0.36</v>
       </c>
       <c r="AM7">
         <v>7.36</v>
@@ -1367,7 +1487,7 @@
         <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C8">
         <v>4.5</v>
@@ -1379,7 +1499,7 @@
         <v>102</v>
       </c>
       <c r="F8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G8">
         <v>824557</v>
@@ -1438,17 +1558,23 @@
       <c r="Y8">
         <v>1.0901</v>
       </c>
+      <c r="Z8">
+        <v>8</v>
+      </c>
       <c r="AA8" t="s">
-        <v>44</v>
+        <v>52</v>
+      </c>
+      <c r="AB8">
+        <v>0.71</v>
       </c>
       <c r="AC8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD8">
         <v>5.21</v>
       </c>
       <c r="AE8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF8">
         <v>0.2033</v>
@@ -1458,6 +1584,18 @@
       </c>
       <c r="AH8">
         <v>0</v>
+      </c>
+      <c r="AI8">
+        <v>2.79</v>
+      </c>
+      <c r="AJ8">
+        <v>2.79</v>
+      </c>
+      <c r="AK8">
+        <v>2.79</v>
+      </c>
+      <c r="AL8">
+        <v>2.79</v>
       </c>
       <c r="AM8">
         <v>5.21</v>
@@ -1468,7 +1606,7 @@
         <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C9">
         <v>3.5</v>
@@ -1480,13 +1618,13 @@
         <v>122</v>
       </c>
       <c r="F9" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G9">
         <v>824557</v>
       </c>
       <c r="H9" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="I9">
         <v>5</v>
@@ -1539,17 +1677,23 @@
       <c r="Y9">
         <v>1.0766</v>
       </c>
+      <c r="Z9">
+        <v>2</v>
+      </c>
       <c r="AA9" t="s">
         <v>44</v>
       </c>
+      <c r="AB9">
+        <v>2.08</v>
+      </c>
       <c r="AC9" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="AD9">
         <v>5.58</v>
       </c>
       <c r="AE9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF9">
         <v>0.1959</v>
@@ -1559,6 +1703,18 @@
       </c>
       <c r="AH9">
         <v>0</v>
+      </c>
+      <c r="AI9">
+        <v>-3.58</v>
+      </c>
+      <c r="AJ9">
+        <v>3.58</v>
+      </c>
+      <c r="AK9">
+        <v>-3.58</v>
+      </c>
+      <c r="AL9">
+        <v>3.58</v>
       </c>
       <c r="AM9">
         <v>5.58</v>
@@ -1569,7 +1725,7 @@
         <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C10">
         <v>7.5</v>
@@ -1581,7 +1737,7 @@
         <v>-150</v>
       </c>
       <c r="F10" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="G10">
         <v>823992</v>
@@ -1640,17 +1796,23 @@
       <c r="Y10">
         <v>1.0953</v>
       </c>
+      <c r="Z10">
+        <v>4</v>
+      </c>
       <c r="AA10" t="s">
         <v>44</v>
       </c>
+      <c r="AB10">
+        <v>2.43</v>
+      </c>
       <c r="AC10" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="AD10">
         <v>9.93</v>
       </c>
       <c r="AE10" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="AF10">
         <v>0.2699</v>
@@ -1660,6 +1822,18 @@
       </c>
       <c r="AH10">
         <v>0</v>
+      </c>
+      <c r="AI10">
+        <v>-5.93</v>
+      </c>
+      <c r="AJ10">
+        <v>5.93</v>
+      </c>
+      <c r="AK10">
+        <v>-5.93</v>
+      </c>
+      <c r="AL10">
+        <v>5.93</v>
       </c>
       <c r="AM10">
         <v>9.93</v>
@@ -1670,7 +1844,7 @@
         <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C11">
         <v>4.5</v>
@@ -1682,13 +1856,13 @@
         <v>-147</v>
       </c>
       <c r="F11" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="G11">
         <v>823992</v>
       </c>
       <c r="H11" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="I11">
         <v>4.3</v>
@@ -1741,17 +1915,23 @@
       <c r="Y11">
         <v>0.88</v>
       </c>
+      <c r="Z11">
+        <v>3</v>
+      </c>
       <c r="AA11" t="s">
         <v>44</v>
       </c>
+      <c r="AB11">
+        <v>-1.84</v>
+      </c>
       <c r="AC11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD11">
         <v>2.66</v>
       </c>
       <c r="AE11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF11">
         <v>0.2079</v>
@@ -1761,6 +1941,18 @@
       </c>
       <c r="AH11">
         <v>0</v>
+      </c>
+      <c r="AI11">
+        <v>0.34</v>
+      </c>
+      <c r="AJ11">
+        <v>0.34</v>
+      </c>
+      <c r="AK11">
+        <v>0.34</v>
+      </c>
+      <c r="AL11">
+        <v>0.34</v>
       </c>
       <c r="AM11">
         <v>2.66</v>
@@ -1771,7 +1963,7 @@
         <v>39</v>
       </c>
       <c r="B12" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C12">
         <v>4.5</v>
@@ -1783,7 +1975,7 @@
         <v>-105</v>
       </c>
       <c r="F12" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="G12">
         <v>825041</v>
@@ -1842,17 +2034,23 @@
       <c r="Y12">
         <v>0.88</v>
       </c>
+      <c r="Z12">
+        <v>6</v>
+      </c>
       <c r="AA12" t="s">
-        <v>44</v>
+        <v>52</v>
+      </c>
+      <c r="AB12">
+        <v>-0.73</v>
       </c>
       <c r="AC12" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="AD12">
         <v>3.77</v>
       </c>
       <c r="AE12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF12">
         <v>0.2294</v>
@@ -1862,6 +2060,18 @@
       </c>
       <c r="AH12">
         <v>0</v>
+      </c>
+      <c r="AI12">
+        <v>2.23</v>
+      </c>
+      <c r="AJ12">
+        <v>2.23</v>
+      </c>
+      <c r="AK12">
+        <v>2.23</v>
+      </c>
+      <c r="AL12">
+        <v>2.23</v>
       </c>
       <c r="AM12">
         <v>3.77</v>
@@ -1872,7 +2082,7 @@
         <v>39</v>
       </c>
       <c r="B13" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C13">
         <v>3.5</v>
@@ -1884,7 +2094,7 @@
         <v>114</v>
       </c>
       <c r="F13" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="G13">
         <v>825041</v>
@@ -1943,17 +2153,23 @@
       <c r="Y13">
         <v>0.9794</v>
       </c>
+      <c r="Z13">
+        <v>4</v>
+      </c>
       <c r="AA13" t="s">
-        <v>44</v>
+        <v>52</v>
+      </c>
+      <c r="AB13">
+        <v>0.26</v>
       </c>
       <c r="AC13" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD13">
         <v>3.76</v>
       </c>
       <c r="AE13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF13">
         <v>0.1552</v>
@@ -1963,6 +2179,18 @@
       </c>
       <c r="AH13">
         <v>0</v>
+      </c>
+      <c r="AI13">
+        <v>0.24</v>
+      </c>
+      <c r="AJ13">
+        <v>0.24</v>
+      </c>
+      <c r="AK13">
+        <v>0.24</v>
+      </c>
+      <c r="AL13">
+        <v>0.24</v>
       </c>
       <c r="AM13">
         <v>3.76</v>
@@ -1973,7 +2201,7 @@
         <v>39</v>
       </c>
       <c r="B14" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C14">
         <v>5.5</v>
@@ -1985,7 +2213,7 @@
         <v>-150</v>
       </c>
       <c r="F14" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="G14">
         <v>823260</v>
@@ -2044,17 +2272,23 @@
       <c r="Y14">
         <v>1.0085</v>
       </c>
+      <c r="Z14">
+        <v>2</v>
+      </c>
       <c r="AA14" t="s">
         <v>44</v>
       </c>
+      <c r="AB14">
+        <v>-0.21</v>
+      </c>
       <c r="AC14" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD14">
         <v>5.29</v>
       </c>
       <c r="AE14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF14">
         <v>0.2549</v>
@@ -2064,6 +2298,18 @@
       </c>
       <c r="AH14">
         <v>0</v>
+      </c>
+      <c r="AI14">
+        <v>-3.29</v>
+      </c>
+      <c r="AJ14">
+        <v>3.29</v>
+      </c>
+      <c r="AK14">
+        <v>-3.29</v>
+      </c>
+      <c r="AL14">
+        <v>3.29</v>
       </c>
       <c r="AM14">
         <v>5.29</v>
@@ -2074,7 +2320,7 @@
         <v>39</v>
       </c>
       <c r="B15" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C15">
         <v>5.5</v>
@@ -2086,7 +2332,7 @@
         <v>-102</v>
       </c>
       <c r="F15" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="G15">
         <v>823260</v>
@@ -2145,17 +2391,23 @@
       <c r="Y15">
         <v>1.0952</v>
       </c>
+      <c r="Z15">
+        <v>5</v>
+      </c>
       <c r="AA15" t="s">
         <v>44</v>
       </c>
+      <c r="AB15">
+        <v>0.78</v>
+      </c>
       <c r="AC15" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="AD15">
         <v>6.28</v>
       </c>
       <c r="AE15" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="AF15">
         <v>0.1964</v>
@@ -2165,6 +2417,18 @@
       </c>
       <c r="AH15">
         <v>0</v>
+      </c>
+      <c r="AI15">
+        <v>-1.28</v>
+      </c>
+      <c r="AJ15">
+        <v>1.28</v>
+      </c>
+      <c r="AK15">
+        <v>-1.28</v>
+      </c>
+      <c r="AL15">
+        <v>1.28</v>
       </c>
       <c r="AM15">
         <v>6.28</v>
@@ -2175,7 +2439,7 @@
         <v>39</v>
       </c>
       <c r="B16" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C16">
         <v>4.5</v>
@@ -2187,7 +2451,7 @@
         <v>-148</v>
       </c>
       <c r="F16" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="G16">
         <v>824964</v>
@@ -2246,17 +2510,23 @@
       <c r="Y16">
         <v>1.0204</v>
       </c>
+      <c r="Z16">
+        <v>7</v>
+      </c>
       <c r="AA16" t="s">
-        <v>44</v>
+        <v>52</v>
+      </c>
+      <c r="AB16">
+        <v>0.15</v>
       </c>
       <c r="AC16" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD16">
         <v>4.65</v>
       </c>
       <c r="AE16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF16">
         <v>0.1997</v>
@@ -2266,6 +2536,18 @@
       </c>
       <c r="AH16">
         <v>0</v>
+      </c>
+      <c r="AI16">
+        <v>2.35</v>
+      </c>
+      <c r="AJ16">
+        <v>2.35</v>
+      </c>
+      <c r="AK16">
+        <v>2.35</v>
+      </c>
+      <c r="AL16">
+        <v>2.35</v>
       </c>
       <c r="AM16">
         <v>4.65</v>
@@ -2276,7 +2558,7 @@
         <v>39</v>
       </c>
       <c r="B17" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C17">
         <v>3.5</v>
@@ -2288,7 +2570,7 @@
         <v>115</v>
       </c>
       <c r="F17" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="G17">
         <v>824964</v>
@@ -2347,17 +2629,23 @@
       <c r="Y17">
         <v>0.9436</v>
       </c>
+      <c r="Z17">
+        <v>3</v>
+      </c>
       <c r="AA17" t="s">
         <v>44</v>
       </c>
+      <c r="AB17">
+        <v>-0.74</v>
+      </c>
       <c r="AC17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD17">
         <v>2.76</v>
       </c>
       <c r="AE17" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF17">
         <v>0.1501</v>
@@ -2367,6 +2655,18 @@
       </c>
       <c r="AH17">
         <v>0</v>
+      </c>
+      <c r="AI17">
+        <v>0.24</v>
+      </c>
+      <c r="AJ17">
+        <v>0.24</v>
+      </c>
+      <c r="AK17">
+        <v>0.24</v>
+      </c>
+      <c r="AL17">
+        <v>0.24</v>
       </c>
       <c r="AM17">
         <v>2.76</v>
@@ -2377,7 +2677,7 @@
         <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C18">
         <v>7.5</v>
@@ -2389,7 +2689,7 @@
         <v>-148</v>
       </c>
       <c r="F18" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G18">
         <v>823097</v>
@@ -2448,17 +2748,23 @@
       <c r="Y18">
         <v>0.9919</v>
       </c>
+      <c r="Z18">
+        <v>4</v>
+      </c>
       <c r="AA18" t="s">
         <v>44</v>
       </c>
+      <c r="AB18">
+        <v>-0.1</v>
+      </c>
       <c r="AC18" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD18">
         <v>7.4</v>
       </c>
       <c r="AE18" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="AF18">
         <v>0.2985</v>
@@ -2468,6 +2774,18 @@
       </c>
       <c r="AH18">
         <v>0</v>
+      </c>
+      <c r="AI18">
+        <v>-3.4</v>
+      </c>
+      <c r="AJ18">
+        <v>3.4</v>
+      </c>
+      <c r="AK18">
+        <v>-3.4</v>
+      </c>
+      <c r="AL18">
+        <v>3.4</v>
       </c>
       <c r="AM18">
         <v>7.4</v>
@@ -2478,7 +2796,7 @@
         <v>39</v>
       </c>
       <c r="B19" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C19">
         <v>6.5</v>
@@ -2490,7 +2808,7 @@
         <v>-140</v>
       </c>
       <c r="F19" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G19">
         <v>823097</v>
@@ -2549,17 +2867,23 @@
       <c r="Y19">
         <v>0.9256</v>
       </c>
+      <c r="Z19">
+        <v>5</v>
+      </c>
       <c r="AA19" t="s">
         <v>44</v>
       </c>
+      <c r="AB19">
+        <v>-2.67</v>
+      </c>
       <c r="AC19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD19">
         <v>3.83</v>
       </c>
       <c r="AE19" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF19">
         <v>0.2511</v>
@@ -2569,6 +2893,18 @@
       </c>
       <c r="AH19">
         <v>0</v>
+      </c>
+      <c r="AI19">
+        <v>1.17</v>
+      </c>
+      <c r="AJ19">
+        <v>1.17</v>
+      </c>
+      <c r="AK19">
+        <v>1.17</v>
+      </c>
+      <c r="AL19">
+        <v>1.17</v>
       </c>
       <c r="AM19">
         <v>3.83</v>
@@ -2579,7 +2915,7 @@
         <v>39</v>
       </c>
       <c r="B20" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C20">
         <v>6.5</v>
@@ -2591,7 +2927,7 @@
         <v>-115</v>
       </c>
       <c r="F20" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="G20">
         <v>823183</v>
@@ -2650,17 +2986,23 @@
       <c r="Y20">
         <v>0.9638</v>
       </c>
+      <c r="Z20">
+        <v>5</v>
+      </c>
       <c r="AA20" t="s">
         <v>44</v>
       </c>
+      <c r="AB20">
+        <v>-0.08</v>
+      </c>
       <c r="AC20" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="AD20">
         <v>6.42</v>
       </c>
       <c r="AE20" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="AF20">
         <v>0.2953</v>
@@ -2670,6 +3012,18 @@
       </c>
       <c r="AH20">
         <v>0</v>
+      </c>
+      <c r="AI20">
+        <v>-1.42</v>
+      </c>
+      <c r="AJ20">
+        <v>1.42</v>
+      </c>
+      <c r="AK20">
+        <v>-1.42</v>
+      </c>
+      <c r="AL20">
+        <v>1.42</v>
       </c>
       <c r="AM20">
         <v>6.42</v>
@@ -2680,7 +3034,7 @@
         <v>39</v>
       </c>
       <c r="B21" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C21">
         <v>4.5</v>
@@ -2692,7 +3046,7 @@
         <v>-117</v>
       </c>
       <c r="F21" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="G21">
         <v>823183</v>
@@ -2751,17 +3105,23 @@
       <c r="Y21">
         <v>1.0671</v>
       </c>
+      <c r="Z21">
+        <v>3</v>
+      </c>
       <c r="AA21" t="s">
         <v>44</v>
       </c>
+      <c r="AB21">
+        <v>0.74</v>
+      </c>
       <c r="AC21" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="AD21">
         <v>5.24</v>
       </c>
       <c r="AE21" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF21">
         <v>0.1533</v>
@@ -2771,6 +3131,18 @@
       </c>
       <c r="AH21">
         <v>0</v>
+      </c>
+      <c r="AI21">
+        <v>-2.24</v>
+      </c>
+      <c r="AJ21">
+        <v>2.24</v>
+      </c>
+      <c r="AK21">
+        <v>-2.24</v>
+      </c>
+      <c r="AL21">
+        <v>2.24</v>
       </c>
       <c r="AM21">
         <v>5.24</v>
@@ -2781,16 +3153,16 @@
         <v>39</v>
       </c>
       <c r="B22" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="F22" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G22">
         <v>824557</v>
       </c>
       <c r="H22" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="I22">
         <v>4.5</v>
@@ -2811,7 +3183,7 @@
         <v>4.44</v>
       </c>
       <c r="S22" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="T22">
         <v>0.2365</v>
@@ -2831,17 +3203,23 @@
       <c r="Y22">
         <v>1.0354</v>
       </c>
+      <c r="Z22">
+        <v>2</v>
+      </c>
       <c r="AA22" t="s">
         <v>44</v>
       </c>
+      <c r="AB22">
+        <v>2.08</v>
+      </c>
       <c r="AC22" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="AD22">
         <v>5.49</v>
       </c>
       <c r="AE22" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF22">
         <v>0.2394</v>
@@ -2851,6 +3229,18 @@
       </c>
       <c r="AH22">
         <v>0</v>
+      </c>
+      <c r="AI22">
+        <v>-3.49</v>
+      </c>
+      <c r="AJ22">
+        <v>3.49</v>
+      </c>
+      <c r="AK22">
+        <v>-3.49</v>
+      </c>
+      <c r="AL22">
+        <v>3.49</v>
       </c>
       <c r="AM22">
         <v>5.49</v>

</xml_diff>